<commit_message>
📊 Отчёт 2026-03-20 13:53 MSK
</commit_message>
<xml_diff>
--- a/logs/excel/fedresurs_2026-03-20.xlsx
+++ b/logs/excel/fedresurs_2026-03-20.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,7 +474,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-20T12:44:32.764997+03:00</t>
+          <t>2026-03-20T13:48:12.474536+03:00</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-20T12:45:03.196179+03:00</t>
+          <t>2026-03-20T13:48:43.673006+03:00</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,53 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-20T12:47:14.176489+03:00</t>
+          <t>2026-03-20T13:50:41.222328+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>7424024375</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ПАО "ЮГК"</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-03-20T13:51:10.986195+03:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7825367884</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>АО "БЕАТОН"</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Нет данных</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-03-20T13:53:11.830808+03:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Отчёт 2026-03-20 14:31 MSK
</commit_message>
<xml_diff>
--- a/logs/excel/fedresurs_2026-03-20.xlsx
+++ b/logs/excel/fedresurs_2026-03-20.xlsx
@@ -474,7 +474,7 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-20T13:48:12.474536+03:00</t>
+          <t>2026-03-20T14:15:11.302790+03:00</t>
         </is>
       </c>
     </row>
@@ -497,7 +497,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-20T13:48:43.673006+03:00</t>
+          <t>2026-03-20T14:16:18.647867+03:00</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-20T13:50:41.222328+03:00</t>
+          <t>2026-03-20T14:29:16.090185+03:00</t>
         </is>
       </c>
     </row>
@@ -543,7 +543,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-03-20T13:51:10.986195+03:00</t>
+          <t>2026-03-20T14:29:41.980732+03:00</t>
         </is>
       </c>
     </row>
@@ -566,7 +566,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-03-20T13:53:11.830808+03:00</t>
+          <t>2026-03-20T14:31:37.132163+03:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Отчёт 2026-03-20 15:41 MSK
</commit_message>
<xml_diff>
--- a/logs/excel/fedresurs_2026-03-20.xlsx
+++ b/logs/excel/fedresurs_2026-03-20.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,11 +449,6 @@
           <t>Публикации</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>timestamp</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -472,11 +467,6 @@
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-03-20T14:53:57.019256+03:00</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -495,11 +485,6 @@
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-03-20T14:54:31.089830+03:00</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -518,11 +503,6 @@
         </is>
       </c>
       <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-03-20T14:56:25.501262+03:00</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -537,15 +517,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Нет данных</t>
+          <t>Сведения о банкротстве:
+Публикации:
+- 10592731 от 10.01.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 04586390 от 09.12.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 04031970 от 24.06.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 03949602 от 27.05.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве</t>
         </is>
       </c>
       <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-03-20T14:56:52.450735+03:00</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -560,15 +540,46 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Нет данных</t>
+          <t>Сведения о банкротстве:
+Публикации:
+- 33724416 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 33724400 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 33724312 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 33724347 от 02.02.2026 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 27696837 от 14.05.2025 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 27212505 от 23.04.2025 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 16349017 от 25.08.2023 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 14495468 от 01.02.2023 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 14160220 от 16.12.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13970684 от 30.11.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13629950 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13607030 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13630478 от 26.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13441177 от 12.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 13441131 от 12.10.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 11223158 от 24.02.2022 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 10314580 от 10.12.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 10069405 от 18.11.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 09924266 от 20.10.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 09755518 от 06.10.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 09708710 от 29.09.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 09242657 от 06.08.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 08703978 от 02.07.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 08704421 от 02.07.2021 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 05799154 от 30.12.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 05704485 от 11.12.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 05616761 от 25.11.2020 Намерение должника обратиться в суд с заявлением о банкротстве
+- 05340350 от 14.10.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 05001697 от 25.06.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 04795597 от 19.03.2020 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 04592154 от 12.12.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 03852906 от 22.04.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 03706767 от 25.02.2019 Намерение кредитора обратиться в суд с заявлением о банкротстве
+- 03196309 от 08.06.2018 Намерение должника обратиться в суд с заявлением о банкротстве
+- 00109989 от 19.08.2015 Намерение должника обратиться в суд с заявлением о банкротстве</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>2026-03-20T14:58:56.914055+03:00</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>